<commit_message>
BOQ Yoseftal y Migdalei: secciones separadas de cableado, instalación, entrenamiento y garantía, con subtotales; precios vacíos
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015wmEUV9EbBvwtcXC6L5hB5
</commit_message>
<xml_diff>
--- a/migdalei/en/BOQ_EN.xlsx
+++ b/migdalei/en/BOQ_EN.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="138">
   <si>
     <t xml:space="preserve">BOQ – BILL OF QUANTITIES AND BUDGET</t>
   </si>
@@ -171,6 +171,9 @@
     <t xml:space="preserve">LCom – apartment radial hub (ceiling)</t>
   </si>
   <si>
+    <t xml:space="preserve">Subtotal</t>
+  </si>
+  <si>
     <t xml:space="preserve">PUBLIC TOILETS</t>
   </si>
   <si>
@@ -249,7 +252,7 @@
     <t xml:space="preserve">nurse desk</t>
   </si>
   <si>
-    <t xml:space="preserve">CABLES (+ reserve, see Cables sheet)</t>
+    <t xml:space="preserve">CABLING (model lengths + reserve, see Cables sheet)</t>
   </si>
   <si>
     <t xml:space="preserve">APT</t>
@@ -276,7 +279,103 @@
     <t xml:space="preserve">Cat6A / Cat7 racks and riser (red)</t>
   </si>
   <si>
-    <t xml:space="preserve">Subtotal</t>
+    <t xml:space="preserve">INSTALLATION</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INS-EQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mounting and connection of devices (panels, lights, pull-cords, PCB/LCom/BoxCom, tablets)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sum of all devices</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INS-CAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cable pulling in tray / ceiling, conduit and labelling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sum of all cabling</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INS-RACK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rack assembly: switch, server, patch panel, UPS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INS-PRG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Programming, commissioning and testing of every call point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">INS-ASB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">As-built drawings and handover protocol</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TRAINING</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-USR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training for nursing / reception staff (daily use)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">session</t>
+  </si>
+  <si>
+    <t xml:space="preserve">per shift</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-TEC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Technical training for maintenance / IT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TR-DOC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">User and technical manuals (ES / EN / HE)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WARRANTY AND SERVICE</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAR-EQ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Equipment warranty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">year</t>
+  </si>
+  <si>
+    <t xml:space="preserve">as per manufacturer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GAR-INS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Installation and workmanship warranty</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MNT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preventive maintenance and technical support (optional)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">optional</t>
   </si>
   <si>
     <t xml:space="preserve">Subtotal incl. contingency</t>
@@ -412,7 +511,7 @@
     <numFmt numFmtId="169" formatCode="0&quot; m&quot;"/>
     <numFmt numFmtId="170" formatCode="0.0"/>
   </numFmts>
-  <fonts count="15">
+  <fonts count="16">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -487,6 +586,14 @@
     <font>
       <sz val="10"/>
       <color rgb="FF008000"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <i val="true"/>
+      <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -593,7 +700,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -658,10 +765,22 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -674,7 +793,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -682,16 +801,12 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="10" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -978,7 +1093,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H35"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1187,85 +1302,42 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="9" t="s">
+      <c r="F15" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="B15" s="9"/>
-      <c r="C15" s="9"/>
-      <c r="D15" s="9"/>
-      <c r="E15" s="9"/>
-      <c r="F15" s="9"/>
-      <c r="G15" s="9"/>
-      <c r="H15" s="9"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="10" t="n">
+      <c r="G15" s="17" t="n">
+        <f aca="false">SUM(G11:G14)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="9" t="s">
+        <v>30</v>
+      </c>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="10" t="n">
         <v>5</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B18" s="11" t="s">
         <v>24</v>
       </c>
-      <c r="C16" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D16" s="10" t="s">
+      <c r="C18" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="D18" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E16" s="13" t="n">
+      <c r="E18" s="13" t="n">
         <f aca="false">'Quantities per level'!F12</f>
         <v>10</v>
-      </c>
-      <c r="F16" s="14"/>
-      <c r="G16" s="15" t="n">
-        <f aca="false">E16*F16</f>
-        <v>0</v>
-      </c>
-      <c r="H16" s="12" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="10" t="n">
-        <v>6</v>
-      </c>
-      <c r="B17" s="11" t="s">
-        <v>32</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D17" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E17" s="13" t="n">
-        <f aca="false">'Quantities per level'!F13</f>
-        <v>10</v>
-      </c>
-      <c r="F17" s="14"/>
-      <c r="G17" s="15" t="n">
-        <f aca="false">E17*F17</f>
-        <v>0</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="10" t="n">
-        <v>7</v>
-      </c>
-      <c r="B18" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="C18" s="12" t="s">
-        <v>35</v>
-      </c>
-      <c r="D18" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E18" s="13" t="n">
-        <f aca="false">'Quantities per level'!F14</f>
-        <v>9</v>
       </c>
       <c r="F18" s="14"/>
       <c r="G18" s="15" t="n">
@@ -1273,37 +1345,51 @@
         <v>0</v>
       </c>
       <c r="H18" s="12" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B19" s="9"/>
-      <c r="C19" s="9"/>
-      <c r="D19" s="9"/>
-      <c r="E19" s="9"/>
-      <c r="F19" s="9"/>
-      <c r="G19" s="9"/>
-      <c r="H19" s="9"/>
+      <c r="A19" s="10" t="n">
+        <v>6</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="D19" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E19" s="13" t="n">
+        <f aca="false">'Quantities per level'!F13</f>
+        <v>10</v>
+      </c>
+      <c r="F19" s="14"/>
+      <c r="G19" s="15" t="n">
+        <f aca="false">E19*F19</f>
+        <v>0</v>
+      </c>
+      <c r="H19" s="12" t="s">
+        <v>35</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="C20" s="12" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="D20" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E20" s="13" t="n">
-        <f aca="false">'Quantities per level'!F16</f>
-        <v>17</v>
+        <f aca="false">'Quantities per level'!F14</f>
+        <v>9</v>
       </c>
       <c r="F20" s="14"/>
       <c r="G20" s="15" t="n">
@@ -1311,103 +1397,46 @@
         <v>0</v>
       </c>
       <c r="H20" s="12" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="B21" s="11" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>42</v>
-      </c>
-      <c r="D21" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E21" s="13" t="n">
-        <f aca="false">'Quantities per level'!F17</f>
-        <v>9</v>
-      </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="15" t="n">
-        <f aca="false">E21*F21</f>
-        <v>0</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10" t="n">
-        <v>10</v>
-      </c>
-      <c r="B22" s="11" t="s">
-        <v>44</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="D22" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E22" s="13" t="n">
-        <f aca="false">'Quantities per level'!F18</f>
-        <v>8</v>
-      </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="15" t="n">
-        <f aca="false">E22*F22</f>
-        <v>0</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>46</v>
+      <c r="F21" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G21" s="17" t="n">
+        <f aca="false">SUM(G18:G20)</f>
+        <v>0</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10" t="n">
-        <v>11</v>
-      </c>
-      <c r="B23" s="11" t="s">
-        <v>47</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="D23" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="E23" s="13" t="n">
-        <f aca="false">'Quantities per level'!F19</f>
-        <v>1</v>
-      </c>
-      <c r="F23" s="14"/>
-      <c r="G23" s="15" t="n">
-        <f aca="false">E23*F23</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>49</v>
-      </c>
+      <c r="A23" s="9" t="s">
+        <v>38</v>
+      </c>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="10" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D24" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E24" s="13" t="n">
-        <f aca="false">'Quantities per level'!F20</f>
-        <v>1</v>
+        <f aca="false">'Quantities per level'!F16</f>
+        <v>17</v>
       </c>
       <c r="F24" s="14"/>
       <c r="G24" s="15" t="n">
@@ -1415,25 +1444,25 @@
         <v>0</v>
       </c>
       <c r="H24" s="12" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="10" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>52</v>
+        <v>42</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>53</v>
+        <v>43</v>
       </c>
       <c r="D25" s="10" t="s">
         <v>19</v>
       </c>
       <c r="E25" s="13" t="n">
-        <f aca="false">'Quantities per level'!F21</f>
-        <v>1</v>
+        <f aca="false">'Quantities per level'!F17</f>
+        <v>9</v>
       </c>
       <c r="F25" s="14"/>
       <c r="G25" s="15" t="n">
@@ -1441,37 +1470,51 @@
         <v>0</v>
       </c>
       <c r="H25" s="12" t="s">
-        <v>54</v>
+        <v>44</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="9" t="s">
-        <v>55</v>
-      </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9"/>
-      <c r="D26" s="9"/>
-      <c r="E26" s="9"/>
-      <c r="F26" s="9"/>
-      <c r="G26" s="9"/>
-      <c r="H26" s="9"/>
+      <c r="A26" s="10" t="n">
+        <v>10</v>
+      </c>
+      <c r="B26" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="13" t="n">
+        <f aca="false">'Quantities per level'!F18</f>
+        <v>8</v>
+      </c>
+      <c r="F26" s="14"/>
+      <c r="G26" s="15" t="n">
+        <f aca="false">E26*F26</f>
+        <v>0</v>
+      </c>
+      <c r="H26" s="12" t="s">
+        <v>47</v>
+      </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="10" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="C27" s="12" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="D27" s="10" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="E27" s="13" t="n">
-        <f aca="false">Cables!G8</f>
-        <v>1700</v>
+        <f aca="false">'Quantities per level'!F19</f>
+        <v>1</v>
       </c>
       <c r="F27" s="14"/>
       <c r="G27" s="15" t="n">
@@ -1479,25 +1522,25 @@
         <v>0</v>
       </c>
       <c r="H27" s="12" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="10" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>60</v>
+        <v>51</v>
       </c>
       <c r="C28" s="12" t="s">
-        <v>61</v>
+        <v>52</v>
       </c>
       <c r="D28" s="10" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="E28" s="13" t="n">
-        <f aca="false">Cables!G9</f>
-        <v>750</v>
+        <f aca="false">'Quantities per level'!F20</f>
+        <v>1</v>
       </c>
       <c r="F28" s="14"/>
       <c r="G28" s="15" t="n">
@@ -1505,25 +1548,25 @@
         <v>0</v>
       </c>
       <c r="H28" s="12" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="10" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>62</v>
+        <v>53</v>
       </c>
       <c r="C29" s="12" t="s">
-        <v>63</v>
+        <v>54</v>
       </c>
       <c r="D29" s="10" t="s">
-        <v>58</v>
+        <v>19</v>
       </c>
       <c r="E29" s="13" t="n">
-        <f aca="false">Cables!G10</f>
-        <v>130</v>
+        <f aca="false">'Quantities per level'!F21</f>
+        <v>1</v>
       </c>
       <c r="F29" s="14"/>
       <c r="G29" s="15" t="n">
@@ -1531,61 +1574,500 @@
         <v>0</v>
       </c>
       <c r="H29" s="12" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F30" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G30" s="17" t="n">
+        <f aca="false">SUM(G24:G29)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="10" t="n">
+        <v>14</v>
+      </c>
+      <c r="B33" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="D33" s="10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F31" s="4" t="s">
+      <c r="E33" s="13" t="n">
+        <f aca="false">Cables!G8</f>
+        <v>1700</v>
+      </c>
+      <c r="F33" s="14"/>
+      <c r="G33" s="15" t="n">
+        <f aca="false">E33*F33</f>
+        <v>0</v>
+      </c>
+      <c r="H33" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E34" s="13" t="n">
+        <f aca="false">Cables!G9</f>
+        <v>750</v>
+      </c>
+      <c r="F34" s="14"/>
+      <c r="G34" s="15" t="n">
+        <f aca="false">E34*F34</f>
+        <v>0</v>
+      </c>
+      <c r="H34" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="10" t="n">
+        <v>16</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="C35" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="G31" s="16" t="n">
-        <f aca="false">SUM(G10:G29)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F32" s="4" t="s">
+      <c r="D35" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E35" s="13" t="n">
+        <f aca="false">Cables!G10</f>
+        <v>130</v>
+      </c>
+      <c r="F35" s="14"/>
+      <c r="G35" s="15" t="n">
+        <f aca="false">E35*F35</f>
+        <v>0</v>
+      </c>
+      <c r="H35" s="12" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F36" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G36" s="17" t="n">
+        <f aca="false">SUM(G33:G35)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="9" t="s">
+        <v>65</v>
+      </c>
+      <c r="B38" s="9"/>
+      <c r="C38" s="9"/>
+      <c r="D38" s="9"/>
+      <c r="E38" s="9"/>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+    </row>
+    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B39" s="11" t="s">
+        <v>66</v>
+      </c>
+      <c r="C39" s="12" t="s">
+        <v>67</v>
+      </c>
+      <c r="D39" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E39" s="18" t="n">
+        <f aca="false">E11+E12+E13+E14+E18+E19+E20+E24+E29</f>
+        <v>319</v>
+      </c>
+      <c r="F39" s="14"/>
+      <c r="G39" s="15" t="n">
+        <f aca="false">E39*F39</f>
+        <v>0</v>
+      </c>
+      <c r="H39" s="12" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B40" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="C40" s="12" t="s">
+        <v>70</v>
+      </c>
+      <c r="D40" s="10" t="s">
+        <v>59</v>
+      </c>
+      <c r="E40" s="18" t="n">
+        <f aca="false">E33+E34+E35</f>
+        <v>2580</v>
+      </c>
+      <c r="F40" s="14"/>
+      <c r="G40" s="15" t="n">
+        <f aca="false">E40*F40</f>
+        <v>0</v>
+      </c>
+      <c r="H40" s="12" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D41" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E41" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="14"/>
+      <c r="G41" s="15" t="n">
+        <f aca="false">E41*F41</f>
+        <v>0</v>
+      </c>
+      <c r="H41" s="12"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="10" t="n">
+        <v>20</v>
+      </c>
+      <c r="B42" s="11" t="s">
+        <v>75</v>
+      </c>
+      <c r="C42" s="12" t="s">
+        <v>76</v>
+      </c>
+      <c r="D42" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E42" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" s="14"/>
+      <c r="G42" s="15" t="n">
+        <f aca="false">E42*F42</f>
+        <v>0</v>
+      </c>
+      <c r="H42" s="12"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="B43" s="11" t="s">
+        <v>77</v>
+      </c>
+      <c r="C43" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="D43" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E43" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F43" s="14"/>
+      <c r="G43" s="15" t="n">
+        <f aca="false">E43*F43</f>
+        <v>0</v>
+      </c>
+      <c r="H43" s="12"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F44" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G44" s="17" t="n">
+        <f aca="false">SUM(G39:G43)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="B46" s="9"/>
+      <c r="C46" s="9"/>
+      <c r="D46" s="9"/>
+      <c r="E46" s="9"/>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B47" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="C47" s="12" t="s">
+        <v>81</v>
+      </c>
+      <c r="D47" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E47" s="19" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" s="14"/>
+      <c r="G47" s="15" t="n">
+        <f aca="false">E47*F47</f>
+        <v>0</v>
+      </c>
+      <c r="H47" s="12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B48" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="C48" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="D48" s="10" t="s">
+        <v>82</v>
+      </c>
+      <c r="E48" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F48" s="14"/>
+      <c r="G48" s="15" t="n">
+        <f aca="false">E48*F48</f>
+        <v>0</v>
+      </c>
+      <c r="H48" s="12"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="10" t="n">
+        <v>24</v>
+      </c>
+      <c r="B49" s="11" t="s">
+        <v>86</v>
+      </c>
+      <c r="C49" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="D49" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="E49" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" s="14"/>
+      <c r="G49" s="15" t="n">
+        <f aca="false">E49*F49</f>
+        <v>0</v>
+      </c>
+      <c r="H49" s="12"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F50" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G50" s="17" t="n">
+        <f aca="false">SUM(G47:G49)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="9" t="s">
+        <v>88</v>
+      </c>
+      <c r="B52" s="9"/>
+      <c r="C52" s="9"/>
+      <c r="D52" s="9"/>
+      <c r="E52" s="9"/>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B53" s="11" t="s">
+        <v>89</v>
+      </c>
+      <c r="C53" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D53" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E53" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F53" s="14"/>
+      <c r="G53" s="15" t="n">
+        <f aca="false">E53*F53</f>
+        <v>0</v>
+      </c>
+      <c r="H53" s="12" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B54" s="11" t="s">
+        <v>93</v>
+      </c>
+      <c r="C54" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="D54" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E54" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" s="14"/>
+      <c r="G54" s="15" t="n">
+        <f aca="false">E54*F54</f>
+        <v>0</v>
+      </c>
+      <c r="H54" s="12"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B55" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C55" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D55" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="E55" s="19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F55" s="14"/>
+      <c r="G55" s="15" t="n">
+        <f aca="false">E55*F55</f>
+        <v>0</v>
+      </c>
+      <c r="H55" s="12" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F56" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G56" s="17" t="n">
+        <f aca="false">SUM(G53:G55)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F58" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="G58" s="17" t="n">
+        <f aca="false">G15+G21+G30+G36+G44+G50+G56</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F59" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G32" s="15" t="n">
-        <f aca="false">G31*$C$6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F33" s="17" t="s">
-        <v>65</v>
-      </c>
-      <c r="G33" s="16" t="n">
-        <f aca="false">G31+G32</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F34" s="4" t="s">
+      <c r="G59" s="15" t="n">
+        <f aca="false">G58*$C$6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F60" s="20" t="s">
+        <v>98</v>
+      </c>
+      <c r="G60" s="17" t="n">
+        <f aca="false">G58+G59</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F61" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G34" s="15" t="n">
-        <f aca="false">G33*$C$7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F35" s="18" t="s">
-        <v>66</v>
-      </c>
-      <c r="G35" s="19" t="n">
-        <f aca="false">G33+G34</f>
+      <c r="G61" s="15" t="n">
+        <f aca="false">G60*$C$7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F62" s="21" t="s">
+        <v>99</v>
+      </c>
+      <c r="G62" s="22" t="n">
+        <f aca="false">G60+G61</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="8">
     <mergeCell ref="E5:H7"/>
     <mergeCell ref="A10:H10"/>
-    <mergeCell ref="A15:H15"/>
-    <mergeCell ref="A19:H19"/>
-    <mergeCell ref="A26:H26"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A23:H23"/>
+    <mergeCell ref="A32:H32"/>
+    <mergeCell ref="A38:H38"/>
+    <mergeCell ref="A46:H46"/>
+    <mergeCell ref="A52:H52"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1615,19 +2097,19 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>67</v>
+      <c r="A1" s="23" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B3" s="21" t="n">
+        <v>101</v>
+      </c>
+      <c r="B3" s="24" t="n">
         <v>8</v>
       </c>
-      <c r="C3" s="22" t="s">
-        <v>69</v>
+      <c r="C3" s="25" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1638,13 +2120,13 @@
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>70</v>
+        <v>103</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>71</v>
+        <v>104</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>72</v>
+        <v>105</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>14</v>
@@ -1654,11 +2136,11 @@
       <c r="A6" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="B6" s="23"/>
-      <c r="C6" s="23"/>
-      <c r="D6" s="23"/>
-      <c r="E6" s="23"/>
-      <c r="F6" s="23"/>
+      <c r="B6" s="26"/>
+      <c r="C6" s="26"/>
+      <c r="D6" s="26"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="26"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="11" t="s">
@@ -1667,301 +2149,301 @@
       <c r="B7" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="24" t="n">
+      <c r="C7" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="25" t="n">
+      <c r="D7" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E7" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="26" t="n">
+      <c r="E7" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="28" t="n">
         <f aca="false">C7*D7+E7</f>
         <v>32</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>73</v>
+        <v>106</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="C8" s="24" t="n">
+        <v>107</v>
+      </c>
+      <c r="C8" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="25" t="n">
+      <c r="D8" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E8" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="26" t="n">
+      <c r="E8" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="28" t="n">
         <f aca="false">C8*D8+E8</f>
         <v>80</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>75</v>
+        <v>108</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="C9" s="24" t="n">
+        <v>109</v>
+      </c>
+      <c r="C9" s="19" t="n">
         <v>16</v>
       </c>
-      <c r="D9" s="25" t="n">
+      <c r="D9" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E9" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="26" t="n">
+      <c r="E9" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="28" t="n">
         <f aca="false">C9*D9+E9</f>
         <v>128</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C10" s="24" t="n">
+        <v>111</v>
+      </c>
+      <c r="C10" s="19" t="n">
         <v>4</v>
       </c>
-      <c r="D10" s="25" t="n">
+      <c r="D10" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E10" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F10" s="26" t="n">
+      <c r="E10" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="28" t="n">
         <f aca="false">C10*D10+E10</f>
         <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="9" t="s">
-        <v>29</v>
-      </c>
-      <c r="B11" s="23"/>
-      <c r="C11" s="23"/>
-      <c r="D11" s="23"/>
-      <c r="E11" s="23"/>
-      <c r="F11" s="23"/>
+        <v>30</v>
+      </c>
+      <c r="B11" s="26"/>
+      <c r="C11" s="26"/>
+      <c r="D11" s="26"/>
+      <c r="E11" s="26"/>
+      <c r="F11" s="26"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>79</v>
+        <v>112</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>80</v>
-      </c>
-      <c r="C12" s="24" t="n">
+        <v>113</v>
+      </c>
+      <c r="C12" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D12" s="25" t="n">
+      <c r="D12" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E12" s="24" t="n">
+      <c r="E12" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="F12" s="26" t="n">
+      <c r="F12" s="28" t="n">
         <f aca="false">C12*D12+E12</f>
         <v>10</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>81</v>
+        <v>114</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>82</v>
-      </c>
-      <c r="C13" s="24" t="n">
+        <v>115</v>
+      </c>
+      <c r="C13" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D13" s="25" t="n">
+      <c r="D13" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E13" s="24" t="n">
+      <c r="E13" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="28" t="n">
         <f aca="false">C13*D13+E13</f>
         <v>10</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>77</v>
+        <v>110</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="C14" s="24" t="n">
+        <v>116</v>
+      </c>
+      <c r="C14" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D14" s="25" t="n">
+      <c r="D14" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E14" s="24" t="n">
+      <c r="E14" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="28" t="n">
         <f aca="false">C14*D14+E14</f>
         <v>9</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="9" t="s">
-        <v>37</v>
-      </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="23"/>
-      <c r="E15" s="23"/>
-      <c r="F15" s="23"/>
+        <v>38</v>
+      </c>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>84</v>
+        <v>117</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="C16" s="24" t="n">
+        <v>118</v>
+      </c>
+      <c r="C16" s="19" t="n">
         <v>2</v>
       </c>
-      <c r="D16" s="25" t="n">
+      <c r="D16" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E16" s="24" t="n">
+      <c r="E16" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="26" t="n">
+      <c r="F16" s="28" t="n">
         <f aca="false">C16*D16+E16</f>
         <v>17</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>86</v>
+        <v>119</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="C17" s="24" t="n">
+        <v>120</v>
+      </c>
+      <c r="C17" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D17" s="25" t="n">
+      <c r="D17" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E17" s="24" t="n">
+      <c r="E17" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="26" t="n">
+      <c r="F17" s="28" t="n">
         <f aca="false">C17*D17+E17</f>
         <v>9</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="11" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B18" s="12" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="24" t="n">
+        <v>46</v>
+      </c>
+      <c r="C18" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="D18" s="25" t="n">
+      <c r="D18" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E18" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="26" t="n">
+      <c r="E18" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="28" t="n">
         <f aca="false">C18*D18+E18</f>
         <v>8</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B19" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="C19" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="25" t="n">
+        <v>49</v>
+      </c>
+      <c r="C19" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E19" s="24" t="n">
+      <c r="E19" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F19" s="28" t="n">
         <f aca="false">C19*D19+E19</f>
         <v>1</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>88</v>
+        <v>121</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="C20" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="25" t="n">
+        <v>122</v>
+      </c>
+      <c r="C20" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E20" s="24" t="n">
+      <c r="E20" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F20" s="26" t="n">
+      <c r="F20" s="28" t="n">
         <f aca="false">C20*D20+E20</f>
         <v>1</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>90</v>
+        <v>123</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="C21" s="24" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="25" t="n">
+        <v>124</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E21" s="24" t="n">
+      <c r="E21" s="19" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="26" t="n">
+      <c r="F21" s="28" t="n">
         <f aca="false">C21*D21+E21</f>
         <v>1</v>
       </c>
@@ -1994,13 +2476,13 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>92</v>
+      <c r="A1" s="23" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>0.15</v>
@@ -2008,115 +2490,115 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="B4" s="27" t="n">
+        <v>127</v>
+      </c>
+      <c r="B4" s="29" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B5" s="28" t="n">
+        <v>101</v>
+      </c>
+      <c r="B5" s="30" t="n">
         <f aca="false">'Quantities per level'!$B$3</f>
         <v>8</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="29" t="s">
+      <c r="A7" s="31" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="29" t="s">
+      <c r="B7" s="31" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="29" t="s">
-        <v>95</v>
-      </c>
-      <c r="D7" s="29" t="s">
-        <v>96</v>
-      </c>
-      <c r="E7" s="29" t="s">
-        <v>97</v>
-      </c>
-      <c r="F7" s="29" t="s">
-        <v>93</v>
-      </c>
-      <c r="G7" s="29" t="s">
-        <v>98</v>
+      <c r="C7" s="31" t="s">
+        <v>128</v>
+      </c>
+      <c r="D7" s="31" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" s="31" t="s">
+        <v>130</v>
+      </c>
+      <c r="F7" s="31" t="s">
+        <v>126</v>
+      </c>
+      <c r="G7" s="31" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="30" t="n">
+        <v>58</v>
+      </c>
+      <c r="C8" s="32" t="n">
         <v>183.1</v>
       </c>
-      <c r="D8" s="30" t="n">
+      <c r="D8" s="32" t="n">
         <v>13.2</v>
       </c>
-      <c r="E8" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="31" t="n">
+      <c r="E8" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="33" t="n">
         <f aca="false">$B$3</f>
         <v>0.15</v>
       </c>
-      <c r="G8" s="26" t="n">
+      <c r="G8" s="28" t="n">
         <f aca="false">ROUNDUP((C8*$B$5+D8+E8)*(1+F8)/$B$4,0)*$B$4</f>
         <v>1700</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>61</v>
-      </c>
-      <c r="C9" s="30" t="n">
+        <v>62</v>
+      </c>
+      <c r="C9" s="32" t="n">
         <v>79.9</v>
       </c>
-      <c r="D9" s="30" t="n">
+      <c r="D9" s="32" t="n">
         <v>11.5</v>
       </c>
-      <c r="E9" s="30" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="31" t="n">
+      <c r="E9" s="32" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="33" t="n">
         <f aca="false">$B$3</f>
         <v>0.15</v>
       </c>
-      <c r="G9" s="26" t="n">
+      <c r="G9" s="28" t="n">
         <f aca="false">ROUNDUP((C9*$B$5+D9+E9)*(1+F9)/$B$4,0)*$B$4</f>
         <v>750</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>63</v>
-      </c>
-      <c r="C10" s="30" t="n">
+        <v>64</v>
+      </c>
+      <c r="C10" s="32" t="n">
         <v>7.4</v>
       </c>
-      <c r="D10" s="30" t="n">
+      <c r="D10" s="32" t="n">
         <v>23.6</v>
       </c>
-      <c r="E10" s="30" t="n">
+      <c r="E10" s="32" t="n">
         <v>28.8</v>
       </c>
-      <c r="F10" s="31" t="n">
+      <c r="F10" s="33" t="n">
         <f aca="false">$B$3</f>
         <v>0.15</v>
       </c>
-      <c r="G10" s="26" t="n">
+      <c r="G10" s="28" t="n">
         <f aca="false">ROUNDUP((C10*$B$5+D10+E10)*(1+F10)/$B$4,0)*$B$4</f>
         <v>130</v>
       </c>
@@ -2145,33 +2627,33 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="20" t="s">
-        <v>99</v>
+      <c r="A1" s="23" t="s">
+        <v>132</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="32" t="s">
-        <v>100</v>
+      <c r="A3" s="34" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="32" t="s">
-        <v>101</v>
+      <c r="A4" s="34" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="32" t="s">
-        <v>102</v>
+      <c r="A5" s="34" t="s">
+        <v>135</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="32" t="s">
-        <v>103</v>
+      <c r="A6" s="34" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="32" t="s">
-        <v>104</v>
+      <c r="A7" s="34" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Migdalei: BOQ con sección opcional Seguridad y sensores, manual y tutorial con el paso nuevo; sin códigos provisorios
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015wmEUV9EbBvwtcXC6L5hB5
</commit_message>
<xml_diff>
--- a/migdalei/en/BOQ_EN.xlsx
+++ b/migdalei/en/BOQ_EN.xlsx
@@ -82,7 +82,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="198" uniqueCount="138">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="178">
   <si>
     <t xml:space="preserve">BOQ – BILL OF QUANTITIES AND BUDGET</t>
   </si>
@@ -90,7 +90,7 @@
     <t xml:space="preserve">Migdalei Yam a Tijon – Assisted living · 8 floors + GF · 32 apartments</t>
   </si>
   <si>
-    <t xml:space="preserve">Client: ACE BG · Advantecnia      Date: 23/10/2026</t>
+    <t xml:space="preserve">Client: ACE BG · Advantecnia      Date: 24/10/2026</t>
   </si>
   <si>
     <t xml:space="preserve">Currency</t>
@@ -252,6 +252,132 @@
     <t xml:space="preserve">nurse desk</t>
   </si>
   <si>
+    <t xml:space="preserve">OPTIONAL – SECURITY AND SENSORS (Smart Room, integrated with nurse call; not added to the total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-CAM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">360° IP camera with fall detection + VoIP audio (ceiling)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bedrooms, living rooms, corridor and common room; GF: hall and reception</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-FALL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WiFi fall detector (bathroom ceiling)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 per bathroom</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-ENV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Environment sensor: smoke, temperature, humidity</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-MED</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical-grade under-mattress sensor (pulse, breathing, bed exit)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 per bed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-TAG</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Resident RTLS wristband with SOS button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 per resident (adjust)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-GW</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RTLS gateway (people and asset tracking)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">each floor corridor + GF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-AP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PoE WiFi access point</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-LOCK</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bluetooth smart lock (apartment door)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-LCK-C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PoE Bluetooth lock controller</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 per floor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-ICOM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IP video intercom at the entrance (answered on the desk phone)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GF entrance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-ACC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Access control: PoE controller + card/PIN reader + electromagnetic lock + exit button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">lot</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GF entrance door</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-EXT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Outdoor IP camera (bullet)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">building entrance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-CAB</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cat6 PoE cable for security and sensors (blue) – model length + 15 %</t>
+  </si>
+  <si>
+    <t xml:space="preserve">m</t>
+  </si>
+  <si>
+    <t xml:space="preserve">to the floor PoE switch / GF server</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SR-INS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Installation, integration with nurse call and commissioning</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Optional subtotal</t>
+  </si>
+  <si>
     <t xml:space="preserve">CABLING (model lengths + reserve, see Cables sheet)</t>
   </si>
   <si>
@@ -261,9 +387,6 @@
     <t xml:space="preserve">Cat6 radial inside the apartments (green)</t>
   </si>
   <si>
-    <t xml:space="preserve">m</t>
-  </si>
-  <si>
     <t xml:space="preserve">model length + reserve</t>
   </si>
   <si>
@@ -304,9 +427,6 @@
   </si>
   <si>
     <t xml:space="preserve">Rack assembly: switch, server, patch panel, UPS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">lot</t>
   </si>
   <si>
     <t xml:space="preserve">INS-PRG</t>
@@ -773,11 +893,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1093,7 +1213,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:H62"/>
+  <dimension ref="A1:H79"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -1598,7 +1718,7 @@
       <c r="G32" s="9"/>
       <c r="H32" s="9"/>
     </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="33" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="10" t="n">
         <v>14</v>
       </c>
@@ -1609,11 +1729,11 @@
         <v>58</v>
       </c>
       <c r="D33" s="10" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="E33" s="13" t="n">
-        <f aca="false">Cables!G8</f>
-        <v>1700</v>
+        <f aca="false">'Quantities per level'!F23</f>
+        <v>106</v>
       </c>
       <c r="F33" s="14"/>
       <c r="G33" s="15" t="n">
@@ -1621,7 +1741,7 @@
         <v>0</v>
       </c>
       <c r="H33" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1629,17 +1749,17 @@
         <v>15</v>
       </c>
       <c r="B34" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="C34" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="C34" s="12" t="s">
-        <v>62</v>
-      </c>
       <c r="D34" s="10" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="E34" s="13" t="n">
-        <f aca="false">Cables!G9</f>
-        <v>750</v>
+        <f aca="false">'Quantities per level'!F24</f>
+        <v>64</v>
       </c>
       <c r="F34" s="14"/>
       <c r="G34" s="15" t="n">
@@ -1647,7 +1767,7 @@
         <v>0</v>
       </c>
       <c r="H34" s="12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1661,11 +1781,11 @@
         <v>64</v>
       </c>
       <c r="D35" s="10" t="s">
-        <v>59</v>
+        <v>19</v>
       </c>
       <c r="E35" s="13" t="n">
-        <f aca="false">Cables!G10</f>
-        <v>130</v>
+        <f aca="false">'Quantities per level'!F25</f>
+        <v>32</v>
       </c>
       <c r="F35" s="14"/>
       <c r="G35" s="15" t="n">
@@ -1673,46 +1793,103 @@
         <v>0</v>
       </c>
       <c r="H35" s="12" t="s">
-        <v>60</v>
+        <v>20</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F36" s="16" t="s">
-        <v>29</v>
-      </c>
-      <c r="G36" s="17" t="n">
-        <f aca="false">SUM(G33:G35)</f>
-        <v>0</v>
+      <c r="A36" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="B36" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="C36" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="D36" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E36" s="13" t="n">
+        <f aca="false">'Quantities per level'!F26</f>
+        <v>48</v>
+      </c>
+      <c r="F36" s="14"/>
+      <c r="G36" s="15" t="n">
+        <f aca="false">E36*F36</f>
+        <v>0</v>
+      </c>
+      <c r="H36" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="10" t="n">
+        <v>18</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="C37" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="D37" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E37" s="13" t="n">
+        <f aca="false">'Quantities per level'!F27</f>
+        <v>48</v>
+      </c>
+      <c r="F37" s="14"/>
+      <c r="G37" s="15" t="n">
+        <f aca="false">E37*F37</f>
+        <v>0</v>
+      </c>
+      <c r="H37" s="12" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" s="9"/>
-      <c r="C38" s="9"/>
-      <c r="D38" s="9"/>
-      <c r="E38" s="9"/>
-      <c r="F38" s="9"/>
-      <c r="G38" s="9"/>
-      <c r="H38" s="9"/>
-    </row>
-    <row r="39" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="10" t="n">
+        <v>19</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="C38" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="D38" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E38" s="13" t="n">
+        <f aca="false">'Quantities per level'!F28</f>
+        <v>17</v>
+      </c>
+      <c r="F38" s="14"/>
+      <c r="G38" s="15" t="n">
+        <f aca="false">E38*F38</f>
+        <v>0</v>
+      </c>
+      <c r="H38" s="12" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="10" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B39" s="11" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>67</v>
+        <v>75</v>
       </c>
       <c r="D39" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="E39" s="18" t="n">
-        <f aca="false">E11+E12+E13+E14+E18+E19+E20+E24+E29</f>
-        <v>319</v>
+      <c r="E39" s="13" t="n">
+        <f aca="false">'Quantities per level'!F29</f>
+        <v>17</v>
       </c>
       <c r="F39" s="14"/>
       <c r="G39" s="15" t="n">
@@ -1720,25 +1897,25 @@
         <v>0</v>
       </c>
       <c r="H39" s="12" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="10" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B40" s="11" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D40" s="10" t="s">
-        <v>59</v>
-      </c>
-      <c r="E40" s="18" t="n">
-        <f aca="false">E33+E34+E35</f>
-        <v>2580</v>
+        <v>19</v>
+      </c>
+      <c r="E40" s="13" t="n">
+        <f aca="false">'Quantities per level'!F30</f>
+        <v>32</v>
       </c>
       <c r="F40" s="14"/>
       <c r="G40" s="15" t="n">
@@ -1746,46 +1923,50 @@
         <v>0</v>
       </c>
       <c r="H40" s="12" t="s">
-        <v>71</v>
+        <v>20</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="10" t="n">
+        <v>22</v>
+      </c>
+      <c r="B41" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="C41" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="D41" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B41" s="11" t="s">
-        <v>72</v>
-      </c>
-      <c r="C41" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="D41" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E41" s="19" t="n">
-        <v>1</v>
+      <c r="E41" s="13" t="n">
+        <f aca="false">'Quantities per level'!F31</f>
+        <v>16</v>
       </c>
       <c r="F41" s="14"/>
       <c r="G41" s="15" t="n">
         <f aca="false">E41*F41</f>
         <v>0</v>
       </c>
-      <c r="H41" s="12"/>
+      <c r="H41" s="12" t="s">
+        <v>80</v>
+      </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="10" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B42" s="11" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D42" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E42" s="19" t="n">
+        <v>19</v>
+      </c>
+      <c r="E42" s="13" t="n">
+        <f aca="false">'Quantities per level'!F32</f>
         <v>1</v>
       </c>
       <c r="F42" s="14"/>
@@ -1793,22 +1974,25 @@
         <f aca="false">E42*F42</f>
         <v>0</v>
       </c>
-      <c r="H42" s="12"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="H42" s="12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B43" s="11" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D43" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E43" s="19" t="n">
+        <v>86</v>
+      </c>
+      <c r="E43" s="13" t="n">
+        <f aca="false">'Quantities per level'!F33</f>
         <v>1</v>
       </c>
       <c r="F43" s="14"/>
@@ -1816,258 +2000,577 @@
         <f aca="false">E43*F43</f>
         <v>0</v>
       </c>
-      <c r="H43" s="12"/>
+      <c r="H43" s="12" t="s">
+        <v>87</v>
+      </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F44" s="16" t="s">
+      <c r="A44" s="10" t="n">
+        <v>25</v>
+      </c>
+      <c r="B44" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="C44" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="D44" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E44" s="13" t="n">
+        <f aca="false">'Quantities per level'!F34</f>
+        <v>1</v>
+      </c>
+      <c r="F44" s="14"/>
+      <c r="G44" s="15" t="n">
+        <f aca="false">E44*F44</f>
+        <v>0</v>
+      </c>
+      <c r="H44" s="12" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="10" t="n">
+        <v>26</v>
+      </c>
+      <c r="B45" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="C45" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="D45" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E45" s="13" t="n">
+        <f aca="false">'Quantities per level'!F35</f>
+        <v>2670</v>
+      </c>
+      <c r="F45" s="14"/>
+      <c r="G45" s="15" t="n">
+        <f aca="false">E45*F45</f>
+        <v>0</v>
+      </c>
+      <c r="H45" s="12" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="10" t="n">
+        <v>27</v>
+      </c>
+      <c r="B46" s="11" t="s">
+        <v>95</v>
+      </c>
+      <c r="C46" s="12" t="s">
+        <v>96</v>
+      </c>
+      <c r="D46" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E46" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F46" s="14"/>
+      <c r="G46" s="15" t="n">
+        <f aca="false">E46*F46</f>
+        <v>0</v>
+      </c>
+      <c r="H46" s="12"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F47" s="16" t="s">
+        <v>97</v>
+      </c>
+      <c r="G47" s="17" t="n">
+        <f aca="false">SUM(G33:G46)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="9" t="s">
+        <v>98</v>
+      </c>
+      <c r="B49" s="9"/>
+      <c r="C49" s="9"/>
+      <c r="D49" s="9"/>
+      <c r="E49" s="9"/>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="n">
+        <v>28</v>
+      </c>
+      <c r="B50" s="11" t="s">
+        <v>99</v>
+      </c>
+      <c r="C50" s="12" t="s">
+        <v>100</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E50" s="13" t="n">
+        <f aca="false">Cables!G8</f>
+        <v>1700</v>
+      </c>
+      <c r="F50" s="14"/>
+      <c r="G50" s="15" t="n">
+        <f aca="false">E50*F50</f>
+        <v>0</v>
+      </c>
+      <c r="H50" s="12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="10" t="n">
         <v>29</v>
       </c>
-      <c r="G44" s="17" t="n">
-        <f aca="false">SUM(G39:G43)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="9" t="s">
-        <v>79</v>
-      </c>
-      <c r="B46" s="9"/>
-      <c r="C46" s="9"/>
-      <c r="D46" s="9"/>
-      <c r="E46" s="9"/>
-      <c r="F46" s="9"/>
-      <c r="G46" s="9"/>
-      <c r="H46" s="9"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="B47" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="C47" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="D47" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="E47" s="19" t="n">
+      <c r="B51" s="11" t="s">
+        <v>102</v>
+      </c>
+      <c r="C51" s="12" t="s">
+        <v>103</v>
+      </c>
+      <c r="D51" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E51" s="13" t="n">
+        <f aca="false">Cables!G9</f>
+        <v>750</v>
+      </c>
+      <c r="F51" s="14"/>
+      <c r="G51" s="15" t="n">
+        <f aca="false">E51*F51</f>
+        <v>0</v>
+      </c>
+      <c r="H51" s="12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="10" t="n">
+        <v>30</v>
+      </c>
+      <c r="B52" s="11" t="s">
+        <v>104</v>
+      </c>
+      <c r="C52" s="12" t="s">
+        <v>105</v>
+      </c>
+      <c r="D52" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E52" s="13" t="n">
+        <f aca="false">Cables!G10</f>
+        <v>130</v>
+      </c>
+      <c r="F52" s="14"/>
+      <c r="G52" s="15" t="n">
+        <f aca="false">E52*F52</f>
+        <v>0</v>
+      </c>
+      <c r="H52" s="12" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F53" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G53" s="17" t="n">
+        <f aca="false">SUM(G50:G52)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="B55" s="9"/>
+      <c r="C55" s="9"/>
+      <c r="D55" s="9"/>
+      <c r="E55" s="9"/>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+    </row>
+    <row r="56" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="10" t="n">
+        <v>31</v>
+      </c>
+      <c r="B56" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C56" s="12" t="s">
+        <v>108</v>
+      </c>
+      <c r="D56" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="E56" s="19" t="n">
+        <f aca="false">E11+E12+E13+E14+E18+E19+E20+E24+E29</f>
+        <v>319</v>
+      </c>
+      <c r="F56" s="14"/>
+      <c r="G56" s="15" t="n">
+        <f aca="false">E56*F56</f>
+        <v>0</v>
+      </c>
+      <c r="H56" s="12" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B57" s="11" t="s">
+        <v>110</v>
+      </c>
+      <c r="C57" s="12" t="s">
+        <v>111</v>
+      </c>
+      <c r="D57" s="10" t="s">
+        <v>93</v>
+      </c>
+      <c r="E57" s="19" t="n">
+        <f aca="false">E50+E51+E52</f>
+        <v>2580</v>
+      </c>
+      <c r="F57" s="14"/>
+      <c r="G57" s="15" t="n">
+        <f aca="false">E57*F57</f>
+        <v>0</v>
+      </c>
+      <c r="H57" s="12" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="10" t="n">
+        <v>33</v>
+      </c>
+      <c r="B58" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C58" s="12" t="s">
+        <v>114</v>
+      </c>
+      <c r="D58" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E58" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" s="14"/>
+      <c r="G58" s="15" t="n">
+        <f aca="false">E58*F58</f>
+        <v>0</v>
+      </c>
+      <c r="H58" s="12"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="10" t="n">
+        <v>34</v>
+      </c>
+      <c r="B59" s="11" t="s">
+        <v>115</v>
+      </c>
+      <c r="C59" s="12" t="s">
+        <v>116</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E59" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="14"/>
+      <c r="G59" s="15" t="n">
+        <f aca="false">E59*F59</f>
+        <v>0</v>
+      </c>
+      <c r="H59" s="12"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="10" t="n">
+        <v>35</v>
+      </c>
+      <c r="B60" s="11" t="s">
+        <v>117</v>
+      </c>
+      <c r="C60" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="D60" s="10" t="s">
+        <v>86</v>
+      </c>
+      <c r="E60" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F60" s="14"/>
+      <c r="G60" s="15" t="n">
+        <f aca="false">E60*F60</f>
+        <v>0</v>
+      </c>
+      <c r="H60" s="12"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F61" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="G61" s="17" t="n">
+        <f aca="false">SUM(G56:G60)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="9" t="s">
+        <v>119</v>
+      </c>
+      <c r="B63" s="9"/>
+      <c r="C63" s="9"/>
+      <c r="D63" s="9"/>
+      <c r="E63" s="9"/>
+      <c r="F63" s="9"/>
+      <c r="G63" s="9"/>
+      <c r="H63" s="9"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="10" t="n">
+        <v>36</v>
+      </c>
+      <c r="B64" s="11" t="s">
+        <v>120</v>
+      </c>
+      <c r="C64" s="12" t="s">
+        <v>121</v>
+      </c>
+      <c r="D64" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="E64" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="F47" s="14"/>
-      <c r="G47" s="15" t="n">
-        <f aca="false">E47*F47</f>
-        <v>0</v>
-      </c>
-      <c r="H47" s="12" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="10" t="n">
-        <v>23</v>
-      </c>
-      <c r="B48" s="11" t="s">
-        <v>84</v>
-      </c>
-      <c r="C48" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="D48" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="E48" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F48" s="14"/>
-      <c r="G48" s="15" t="n">
-        <f aca="false">E48*F48</f>
-        <v>0</v>
-      </c>
-      <c r="H48" s="12"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B49" s="11" t="s">
+      <c r="F64" s="14"/>
+      <c r="G64" s="15" t="n">
+        <f aca="false">E64*F64</f>
+        <v>0</v>
+      </c>
+      <c r="H64" s="12" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="10" t="n">
+        <v>37</v>
+      </c>
+      <c r="B65" s="11" t="s">
+        <v>124</v>
+      </c>
+      <c r="C65" s="12" t="s">
+        <v>125</v>
+      </c>
+      <c r="D65" s="10" t="s">
+        <v>122</v>
+      </c>
+      <c r="E65" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F65" s="14"/>
+      <c r="G65" s="15" t="n">
+        <f aca="false">E65*F65</f>
+        <v>0</v>
+      </c>
+      <c r="H65" s="12"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="10" t="n">
+        <v>38</v>
+      </c>
+      <c r="B66" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="C66" s="12" t="s">
+        <v>127</v>
+      </c>
+      <c r="D66" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="C49" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="D49" s="10" t="s">
-        <v>74</v>
-      </c>
-      <c r="E49" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F49" s="14"/>
-      <c r="G49" s="15" t="n">
-        <f aca="false">E49*F49</f>
-        <v>0</v>
-      </c>
-      <c r="H49" s="12"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F50" s="16" t="s">
+      <c r="E66" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="14"/>
+      <c r="G66" s="15" t="n">
+        <f aca="false">E66*F66</f>
+        <v>0</v>
+      </c>
+      <c r="H66" s="12"/>
+    </row>
+    <row r="67" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F67" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="G50" s="17" t="n">
-        <f aca="false">SUM(G47:G49)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="9" t="s">
-        <v>88</v>
-      </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9"/>
-      <c r="D52" s="9"/>
-      <c r="E52" s="9"/>
-      <c r="F52" s="9"/>
-      <c r="G52" s="9"/>
-      <c r="H52" s="9"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="10" t="n">
-        <v>25</v>
-      </c>
-      <c r="B53" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="C53" s="12" t="s">
-        <v>90</v>
-      </c>
-      <c r="D53" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E53" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F53" s="14"/>
-      <c r="G53" s="15" t="n">
-        <f aca="false">E53*F53</f>
-        <v>0</v>
-      </c>
-      <c r="H53" s="12" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="10" t="n">
-        <v>26</v>
-      </c>
-      <c r="B54" s="11" t="s">
-        <v>93</v>
-      </c>
-      <c r="C54" s="12" t="s">
-        <v>94</v>
-      </c>
-      <c r="D54" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E54" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F54" s="14"/>
-      <c r="G54" s="15" t="n">
-        <f aca="false">E54*F54</f>
-        <v>0</v>
-      </c>
-      <c r="H54" s="12"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="B55" s="11" t="s">
-        <v>95</v>
-      </c>
-      <c r="C55" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="D55" s="10" t="s">
-        <v>91</v>
-      </c>
-      <c r="E55" s="19" t="n">
-        <v>1</v>
-      </c>
-      <c r="F55" s="14"/>
-      <c r="G55" s="15" t="n">
-        <f aca="false">E55*F55</f>
-        <v>0</v>
-      </c>
-      <c r="H55" s="12" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F56" s="16" t="s">
+      <c r="G67" s="17" t="n">
+        <f aca="false">SUM(G64:G66)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="9" t="s">
+        <v>128</v>
+      </c>
+      <c r="B69" s="9"/>
+      <c r="C69" s="9"/>
+      <c r="D69" s="9"/>
+      <c r="E69" s="9"/>
+      <c r="F69" s="9"/>
+      <c r="G69" s="9"/>
+      <c r="H69" s="9"/>
+    </row>
+    <row r="70" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B70" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="C70" s="12" t="s">
+        <v>130</v>
+      </c>
+      <c r="D70" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E70" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" s="14"/>
+      <c r="G70" s="15" t="n">
+        <f aca="false">E70*F70</f>
+        <v>0</v>
+      </c>
+      <c r="H70" s="12" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="10" t="n">
+        <v>40</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>133</v>
+      </c>
+      <c r="C71" s="12" t="s">
+        <v>134</v>
+      </c>
+      <c r="D71" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E71" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F71" s="14"/>
+      <c r="G71" s="15" t="n">
+        <f aca="false">E71*F71</f>
+        <v>0</v>
+      </c>
+      <c r="H71" s="12"/>
+    </row>
+    <row r="72" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="10" t="n">
+        <v>41</v>
+      </c>
+      <c r="B72" s="11" t="s">
+        <v>135</v>
+      </c>
+      <c r="C72" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="D72" s="10" t="s">
+        <v>131</v>
+      </c>
+      <c r="E72" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F72" s="14"/>
+      <c r="G72" s="15" t="n">
+        <f aca="false">E72*F72</f>
+        <v>0</v>
+      </c>
+      <c r="H72" s="12" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F73" s="16" t="s">
         <v>29</v>
       </c>
-      <c r="G56" s="17" t="n">
-        <f aca="false">SUM(G53:G55)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F58" s="4" t="s">
+      <c r="G73" s="17" t="n">
+        <f aca="false">SUM(G70:G72)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F75" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="G58" s="17" t="n">
-        <f aca="false">G15+G21+G30+G36+G44+G50+G56</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F59" s="4" t="s">
+      <c r="G75" s="17" t="n">
+        <f aca="false">G15+G21+G30+G53+G61+G67+G73</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F76" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="G59" s="15" t="n">
-        <f aca="false">G58*$C$6</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F60" s="20" t="s">
-        <v>98</v>
-      </c>
-      <c r="G60" s="17" t="n">
-        <f aca="false">G58+G59</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F61" s="4" t="s">
+      <c r="G76" s="15" t="n">
+        <f aca="false">G75*$C$6</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F77" s="20" t="s">
+        <v>138</v>
+      </c>
+      <c r="G77" s="17" t="n">
+        <f aca="false">G75+G76</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F78" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="G61" s="15" t="n">
-        <f aca="false">G60*$C$7</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="F62" s="21" t="s">
-        <v>99</v>
-      </c>
-      <c r="G62" s="22" t="n">
-        <f aca="false">G60+G61</f>
+      <c r="G78" s="15" t="n">
+        <f aca="false">G77*$C$7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="F79" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="G79" s="22" t="n">
+        <f aca="false">G77+G78</f>
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="E5:H7"/>
     <mergeCell ref="A10:H10"/>
     <mergeCell ref="A17:H17"/>
     <mergeCell ref="A23:H23"/>
     <mergeCell ref="A32:H32"/>
-    <mergeCell ref="A38:H38"/>
-    <mergeCell ref="A46:H46"/>
-    <mergeCell ref="A52:H52"/>
+    <mergeCell ref="A49:H49"/>
+    <mergeCell ref="A55:H55"/>
+    <mergeCell ref="A63:H63"/>
+    <mergeCell ref="A69:H69"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2085,7 +2588,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F21"/>
+  <dimension ref="A1:F35"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="10"/>
@@ -2098,18 +2601,18 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>100</v>
+        <v>140</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>101</v>
+        <v>141</v>
       </c>
       <c r="B3" s="24" t="n">
         <v>8</v>
       </c>
       <c r="C3" s="25" t="s">
-        <v>102</v>
+        <v>142</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2120,13 +2623,13 @@
         <v>10</v>
       </c>
       <c r="C5" s="8" t="s">
-        <v>103</v>
+        <v>143</v>
       </c>
       <c r="D5" s="8" t="s">
-        <v>104</v>
+        <v>144</v>
       </c>
       <c r="E5" s="8" t="s">
-        <v>105</v>
+        <v>145</v>
       </c>
       <c r="F5" s="8" t="s">
         <v>14</v>
@@ -2149,14 +2652,14 @@
       <c r="B7" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="C7" s="19" t="n">
+      <c r="C7" s="18" t="n">
         <v>4</v>
       </c>
       <c r="D7" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F7" s="28" t="n">
@@ -2166,19 +2669,19 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>106</v>
+        <v>146</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="C8" s="19" t="n">
+        <v>147</v>
+      </c>
+      <c r="C8" s="18" t="n">
         <v>10</v>
       </c>
       <c r="D8" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E8" s="19" t="n">
+      <c r="E8" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F8" s="28" t="n">
@@ -2188,19 +2691,19 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>108</v>
+        <v>148</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="C9" s="19" t="n">
+        <v>149</v>
+      </c>
+      <c r="C9" s="18" t="n">
         <v>16</v>
       </c>
       <c r="D9" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F9" s="28" t="n">
@@ -2210,19 +2713,19 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C10" s="19" t="n">
+        <v>151</v>
+      </c>
+      <c r="C10" s="18" t="n">
         <v>4</v>
       </c>
       <c r="D10" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E10" s="19" t="n">
+      <c r="E10" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F10" s="28" t="n">
@@ -2242,19 +2745,19 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="11" t="s">
-        <v>112</v>
+        <v>152</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="C12" s="19" t="n">
+        <v>153</v>
+      </c>
+      <c r="C12" s="18" t="n">
         <v>1</v>
       </c>
       <c r="D12" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E12" s="19" t="n">
+      <c r="E12" s="18" t="n">
         <v>2</v>
       </c>
       <c r="F12" s="28" t="n">
@@ -2264,19 +2767,19 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="11" t="s">
-        <v>114</v>
+        <v>154</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C13" s="19" t="n">
+        <v>155</v>
+      </c>
+      <c r="C13" s="18" t="n">
         <v>1</v>
       </c>
       <c r="D13" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="18" t="n">
         <v>2</v>
       </c>
       <c r="F13" s="28" t="n">
@@ -2286,19 +2789,19 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="11" t="s">
-        <v>110</v>
+        <v>150</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="C14" s="19" t="n">
+        <v>156</v>
+      </c>
+      <c r="C14" s="18" t="n">
         <v>1</v>
       </c>
       <c r="D14" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E14" s="19" t="n">
+      <c r="E14" s="18" t="n">
         <v>1</v>
       </c>
       <c r="F14" s="28" t="n">
@@ -2318,19 +2821,19 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="11" t="s">
-        <v>117</v>
+        <v>157</v>
       </c>
       <c r="B16" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C16" s="19" t="n">
+        <v>158</v>
+      </c>
+      <c r="C16" s="18" t="n">
         <v>2</v>
       </c>
       <c r="D16" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E16" s="19" t="n">
+      <c r="E16" s="18" t="n">
         <v>1</v>
       </c>
       <c r="F16" s="28" t="n">
@@ -2340,19 +2843,19 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="11" t="s">
-        <v>119</v>
+        <v>159</v>
       </c>
       <c r="B17" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="C17" s="19" t="n">
+        <v>160</v>
+      </c>
+      <c r="C17" s="18" t="n">
         <v>1</v>
       </c>
       <c r="D17" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E17" s="19" t="n">
+      <c r="E17" s="18" t="n">
         <v>1</v>
       </c>
       <c r="F17" s="28" t="n">
@@ -2367,14 +2870,14 @@
       <c r="B18" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="C18" s="19" t="n">
+      <c r="C18" s="18" t="n">
         <v>1</v>
       </c>
       <c r="D18" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E18" s="19" t="n">
+      <c r="E18" s="18" t="n">
         <v>0</v>
       </c>
       <c r="F18" s="28" t="n">
@@ -2389,14 +2892,14 @@
       <c r="B19" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="C19" s="19" t="n">
+      <c r="C19" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D19" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E19" s="19" t="n">
+      <c r="E19" s="18" t="n">
         <v>1</v>
       </c>
       <c r="F19" s="28" t="n">
@@ -2406,19 +2909,19 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>121</v>
+        <v>161</v>
       </c>
       <c r="B20" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="C20" s="19" t="n">
+        <v>162</v>
+      </c>
+      <c r="C20" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D20" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E20" s="19" t="n">
+      <c r="E20" s="18" t="n">
         <v>1</v>
       </c>
       <c r="F20" s="28" t="n">
@@ -2428,24 +2931,320 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="11" t="s">
-        <v>123</v>
+        <v>163</v>
       </c>
       <c r="B21" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="C21" s="19" t="n">
+        <v>164</v>
+      </c>
+      <c r="C21" s="18" t="n">
         <v>0</v>
       </c>
       <c r="D21" s="27" t="n">
         <f aca="false">$B$3</f>
         <v>8</v>
       </c>
-      <c r="E21" s="19" t="n">
+      <c r="E21" s="18" t="n">
         <v>1</v>
       </c>
       <c r="F21" s="28" t="n">
         <f aca="false">C21*D21+E21</f>
         <v>1</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="9" t="s">
+        <v>56</v>
+      </c>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="26"/>
+      <c r="E22" s="26"/>
+      <c r="F22" s="26"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>57</v>
+      </c>
+      <c r="B23" s="12" t="s">
+        <v>58</v>
+      </c>
+      <c r="C23" s="18" t="n">
+        <v>13</v>
+      </c>
+      <c r="D23" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E23" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="28" t="n">
+        <f aca="false">C23*D23+E23</f>
+        <v>106</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>61</v>
+      </c>
+      <c r="C24" s="18" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E24" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="28" t="n">
+        <f aca="false">C24*D24+E24</f>
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>64</v>
+      </c>
+      <c r="C25" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D25" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E25" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="28" t="n">
+        <f aca="false">C25*D25+E25</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>65</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C26" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D26" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E26" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="28" t="n">
+        <f aca="false">C26*D26+E26</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="18" t="n">
+        <v>6</v>
+      </c>
+      <c r="D27" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E27" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="28" t="n">
+        <f aca="false">C27*D27+E27</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>72</v>
+      </c>
+      <c r="C28" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E28" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="28" t="n">
+        <f aca="false">C28*D28+E28</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>75</v>
+      </c>
+      <c r="C29" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E29" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F29" s="28" t="n">
+        <f aca="false">C29*D29+E29</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="11" t="s">
+        <v>76</v>
+      </c>
+      <c r="B30" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="C30" s="18" t="n">
+        <v>4</v>
+      </c>
+      <c r="D30" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E30" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="28" t="n">
+        <f aca="false">C30*D30+E30</f>
+        <v>32</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="11" t="s">
+        <v>78</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="18" t="n">
+        <v>2</v>
+      </c>
+      <c r="D31" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E31" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="28" t="n">
+        <f aca="false">C31*D31+E31</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="11" t="s">
+        <v>81</v>
+      </c>
+      <c r="B32" s="12" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E32" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F32" s="28" t="n">
+        <f aca="false">C32*D32+E32</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="B33" s="12" t="s">
+        <v>85</v>
+      </c>
+      <c r="C33" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E33" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" s="28" t="n">
+        <f aca="false">C33*D33+E33</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="11" t="s">
+        <v>88</v>
+      </c>
+      <c r="B34" s="12" t="s">
+        <v>89</v>
+      </c>
+      <c r="C34" s="18" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E34" s="18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" s="28" t="n">
+        <f aca="false">C34*D34+E34</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="11" t="s">
+        <v>91</v>
+      </c>
+      <c r="B35" s="12" t="s">
+        <v>92</v>
+      </c>
+      <c r="C35" s="18" t="n">
+        <v>320</v>
+      </c>
+      <c r="D35" s="27" t="n">
+        <f aca="false">$B$3</f>
+        <v>8</v>
+      </c>
+      <c r="E35" s="18" t="n">
+        <v>110</v>
+      </c>
+      <c r="F35" s="28" t="n">
+        <f aca="false">C35*D35+E35</f>
+        <v>2670</v>
       </c>
     </row>
   </sheetData>
@@ -2477,12 +3276,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>125</v>
+        <v>165</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>126</v>
+        <v>166</v>
       </c>
       <c r="B3" s="7" t="n">
         <v>0.15</v>
@@ -2490,7 +3289,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>127</v>
+        <v>167</v>
       </c>
       <c r="B4" s="29" t="n">
         <v>10</v>
@@ -2498,7 +3297,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>101</v>
+        <v>141</v>
       </c>
       <c r="B5" s="30" t="n">
         <f aca="false">'Quantities per level'!$B$3</f>
@@ -2513,27 +3312,27 @@
         <v>10</v>
       </c>
       <c r="C7" s="31" t="s">
-        <v>128</v>
+        <v>168</v>
       </c>
       <c r="D7" s="31" t="s">
-        <v>129</v>
+        <v>169</v>
       </c>
       <c r="E7" s="31" t="s">
-        <v>130</v>
+        <v>170</v>
       </c>
       <c r="F7" s="31" t="s">
-        <v>126</v>
+        <v>166</v>
       </c>
       <c r="G7" s="31" t="s">
-        <v>131</v>
+        <v>171</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>57</v>
+        <v>99</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>58</v>
+        <v>100</v>
       </c>
       <c r="C8" s="32" t="n">
         <v>183.1</v>
@@ -2555,10 +3354,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="11" t="s">
-        <v>61</v>
+        <v>102</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>62</v>
+        <v>103</v>
       </c>
       <c r="C9" s="32" t="n">
         <v>79.9</v>
@@ -2580,10 +3379,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="11" t="s">
-        <v>63</v>
+        <v>104</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>64</v>
+        <v>105</v>
       </c>
       <c r="C10" s="32" t="n">
         <v>7.4</v>
@@ -2628,32 +3427,32 @@
   <sheetData>
     <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="23" t="s">
-        <v>132</v>
+        <v>172</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="34" t="s">
-        <v>133</v>
+        <v>173</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="34" t="s">
-        <v>134</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="34" t="s">
-        <v>135</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="34" t="s">
-        <v>136</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="34" t="s">
-        <v>137</v>
+        <v>177</v>
       </c>
     </row>
   </sheetData>

</xml_diff>